<commit_message>
Updated automatic bill number system
</commit_message>
<xml_diff>
--- a/kavi_stock_management.xlsx
+++ b/kavi_stock_management.xlsx
@@ -5,16 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Documents\KAVI DIGITAL SOLUTIONS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Documents\GITHUB PROJECTS\KAVI DIGITAL SOLUTIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E46C5CE-438E-4483-B426-EFFF2AB31E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{421594D3-C30B-4C42-9849-D3331A39CBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{AE8545F6-6115-465A-900A-E1B06D7DC738}"/>
   </bookViews>
   <sheets>
     <sheet name="STOCK" sheetId="1" r:id="rId1"/>
     <sheet name="BILLING" sheetId="2" r:id="rId2"/>
+    <sheet name="Dashboard" sheetId="3" r:id="rId3"/>
+    <sheet name="BILL HISTORY" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>Product ID</t>
   </si>
@@ -115,6 +117,44 @@
   </si>
   <si>
     <t>Grand   Total</t>
+  </si>
+  <si>
+    <t>KAVI_DIGITAL_SOLUTIONS</t>
+  </si>
+  <si>
+    <t>INVENTORY &amp; BILLING DASHBOARD</t>
+  </si>
+  <si>
+    <t>TOTAL PRODUCTS</t>
+  </si>
+  <si>
+    <t>TOTAL OPENING STOCKS</t>
+  </si>
+  <si>
+    <t>LOW STOCK ITEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BILLING TOTAL </t>
+  </si>
+  <si>
+    <t>PRODUCT 
+NAME</t>
+  </si>
+  <si>
+    <t>AVAILABLE
+ STOCK</t>
+  </si>
+  <si>
+    <t>PREVIOUS BILL NO.</t>
+  </si>
+  <si>
+    <t>DATE</t>
+  </si>
+  <si>
+    <t>CUSTOMER NAME</t>
+  </si>
+  <si>
+    <t>TOTAL AMOUNT</t>
   </si>
 </sst>
 </file>
@@ -124,7 +164,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,6 +189,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="16"/>
       <color theme="1"/>
@@ -156,8 +203,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,6 +240,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -247,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -260,8 +345,49 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -269,17 +395,18 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -300,16 +427,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -323,8 +440,924 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-IN"/>
+              <a:t>AVAILABLE STOCK BY PRODUCT</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="4.9977688623370639E-2"/>
+          <c:y val="0.16125833012887225"/>
+          <c:w val="0.90297462817147855"/>
+          <c:h val="0.72125801983085447"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$B$8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>AVAILABLE
+ STOCK</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$A$9:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Rice</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Oil</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Sugar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Biscuit</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Milk</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Dashboard!$B$9:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2698-442D-838E-C9B3F193C8CF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="951777711"/>
+        <c:axId val="1294242639"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="951777711"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1294242639"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1294242639"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="951777711"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>114734</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>43296</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDFED698-815D-2510-971D-57C34B1DBE2B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -645,7 +1678,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7957E9B2-178C-4DC1-9480-6A763EA0A2B3}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -656,30 +1689,30 @@
     <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -694,18 +1727,18 @@
       </c>
       <c r="E2" s="2">
         <f>SUMIF(BILLING!$A$2:$A$100,B2,BILLING!$B$2:$B$100)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F2" s="2">
         <f>C2-E2</f>
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G2" s="2" t="str">
         <f>IF(F2&lt;=10,"Low Stock","Available")</f>
         <v>Available</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -731,7 +1764,7 @@
         <v>Low Stock</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -757,7 +1790,7 @@
         <v>Available</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -783,7 +1816,7 @@
         <v>Available</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -825,7 +1858,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E686C6A-30B6-4DDD-BCA5-318CCDEC0A0F}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -835,7 +1868,7 @@
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -855,12 +1888,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C2" s="3">
         <f>VLOOKUP(A2,STOCK!$B$2:$D$6,3,FALSE)</f>
@@ -868,16 +1901,16 @@
       </c>
       <c r="D2" s="3">
         <f>B2*C2</f>
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>18</v>
       </c>
       <c r="G2" s="4">
-        <v>1001</v>
+        <v>1002</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -897,10 +1930,10 @@
       </c>
       <c r="G3" s="5">
         <f ca="1">TODAY()</f>
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -915,8 +1948,14 @@
         <f t="shared" si="0"/>
         <v>135</v>
       </c>
+      <c r="F4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -932,21 +1971,207 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:7" ht="30" customHeight="1">
+      <c r="A6" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="10">
+      <c r="B6" s="26"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="8">
         <f>SUM(D2:D5)</f>
-        <v>1545</v>
+        <v>1725</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A6:C6"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B71C015-499C-4361-BBB5-A7AD670E099A}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="20"/>
+      <c r="E4" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="24"/>
+      <c r="G4" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="26.25">
+      <c r="A5" s="13">
+        <f>COUNTA(STOCK!B2:B6)</f>
+        <v>5</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="17">
+        <f>SUM(STOCK!C2:C6)</f>
+        <v>205</v>
+      </c>
+      <c r="D5" s="18"/>
+      <c r="E5" s="21">
+        <f>COUNTIF(STOCK!G2:G6,"Low Stock")</f>
+        <v>1</v>
+      </c>
+      <c r="F5" s="22"/>
+      <c r="G5" s="11">
+        <f>BILLING!D6</f>
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30">
+      <c r="A8" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="10" t="str">
+        <f>STOCK!B2</f>
+        <v>Rice</v>
+      </c>
+      <c r="B9" s="6">
+        <f>STOCK!F2</f>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="10" t="str">
+        <f>STOCK!B3</f>
+        <v>Oil</v>
+      </c>
+      <c r="B10" s="6">
+        <f>STOCK!F3</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="10" t="str">
+        <f>STOCK!B4</f>
+        <v>Sugar</v>
+      </c>
+      <c r="B11" s="6">
+        <f>STOCK!F4</f>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="10" t="str">
+        <f>STOCK!B5</f>
+        <v>Biscuit</v>
+      </c>
+      <c r="B12" s="6">
+        <f>STOCK!F5</f>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="10" t="str">
+        <f>STOCK!B6</f>
+        <v>Milk</v>
+      </c>
+      <c r="B13" s="6">
+        <f>STOCK!F6</f>
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E4:F4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{441715B6-7887-44AE-8FBB-C8711E5B860C}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="30">
+        <v>46311</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>1725</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -961,6 +2186,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBF644B98343FA47BA84AD0FD7E20570" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5b8656e83e5078bfe48c22c6f1684e03">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c1c96588-e0a5-47e1-b0a5-05bf40062dd1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6742b20410aa247db5aa1d93f98ab5a6" ns3:_="">
     <xsd:import namespace="c1c96588-e0a5-47e1-b0a5-05bf40062dd1"/>
@@ -1104,10 +2335,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01VDG6DXESIHUHKSJG3NBYWRPBGIIWDHKI:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9lbGNvdGVkdS1teS5zaGFyZXBvaW50LmNvbS86dTovZy9wZXJzb25hbC9zMDM4NTkzOV9lZHVfZWxjb3RfaW4vSVFDU1FlaDFTU2JiUTR0RjRUSVJZWjFJQVFGTkVvZ0FaT1pMYmduaGpPdWtiUFE"/>
+</scriptIds>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1119,6 +2350,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E746E4-0941-4A77-9C00-A094A552F5FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="c1c96588-e0a5-47e1-b0a5-05bf40062dd1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C788AFB-B7FF-4CFC-A46D-9D7A5DC5A7DA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1136,18 +2383,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E746E4-0941-4A77-9C00-A094A552F5FC}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0626FC7D-512E-47E2-8D36-0526140956A0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="c1c96588-e0a5-47e1-b0a5-05bf40062dd1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Adjusted Bill History column widths
</commit_message>
<xml_diff>
--- a/kavi_stock_management.xlsx
+++ b/kavi_stock_management.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acer\Documents\GITHUB PROJECTS\KAVI DIGITAL SOLUTIONS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{421594D3-C30B-4C42-9849-D3331A39CBAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91F9330-25AB-4767-AA0E-5CBD493D5314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{AE8545F6-6115-465A-900A-E1B06D7DC738}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{AE8545F6-6115-465A-900A-E1B06D7DC738}"/>
   </bookViews>
   <sheets>
     <sheet name="STOCK" sheetId="1" r:id="rId1"/>
@@ -218,7 +218,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -264,6 +264,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -332,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -402,6 +408,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2140,20 +2149,23 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" t="s">
+      <c r="A1" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="31" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>